<commit_message>
Mise à jour automatique des résultats FFBB
</commit_message>
<xml_diff>
--- a/data/rencontres/rencontres.xlsx
+++ b/data/rencontres/rencontres.xlsx
@@ -50,6 +50,33 @@
     <t>Forfait 2</t>
   </si>
   <si>
+    <t>DXU9-8</t>
+  </si>
+  <si>
+    <t>29959</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (5) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST AMAND P H (6) </t>
+  </si>
+  <si>
+    <t>19/09/2026</t>
+  </si>
+  <si>
+    <t>11:00</t>
+  </si>
+  <si>
+    <t>JEAN DEGROS</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Non</t>
+  </si>
+  <si>
     <t>DFU9-8</t>
   </si>
   <si>
@@ -62,19 +89,64 @@
     <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (8) </t>
   </si>
   <si>
-    <t>19/09/2026</t>
-  </si>
-  <si>
     <t>12:30</t>
   </si>
   <si>
     <t>BEATRICE HEISS</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>Non</t>
+    <t>DMU18-2</t>
+  </si>
+  <si>
+    <t>4617</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST AMAND P H (3) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (4) </t>
+  </si>
+  <si>
+    <t>20/09/2026</t>
+  </si>
+  <si>
+    <t>13:00</t>
+  </si>
+  <si>
+    <t>MAURICE HUGOT</t>
+  </si>
+  <si>
+    <t>M9XEW737</t>
+  </si>
+  <si>
+    <t>DMU11-8</t>
+  </si>
+  <si>
+    <t>28402</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ORCHESIEN B C - 2 (3) </t>
+  </si>
+  <si>
+    <t>LEO LAGRANGE</t>
+  </si>
+  <si>
+    <t>WXEC6PRG</t>
+  </si>
+  <si>
+    <t>DMU15-2</t>
+  </si>
+  <si>
+    <t>8961</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ONNAING JA (3) </t>
+  </si>
+  <si>
+    <t>18:30</t>
+  </si>
+  <si>
+    <t>Daniel COLMONT</t>
   </si>
   <si>
     <t>DFU13-2</t>
@@ -92,51 +164,6 @@
     <t>15:30</t>
   </si>
   <si>
-    <t>JEAN DEGROS</t>
-  </si>
-  <si>
-    <t>DMU11-8</t>
-  </si>
-  <si>
-    <t>28402</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ORCHESIEN B C - 2 (3) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (4) </t>
-  </si>
-  <si>
-    <t>11:00</t>
-  </si>
-  <si>
-    <t>LEO LAGRANGE</t>
-  </si>
-  <si>
-    <t>WXEC6PRG</t>
-  </si>
-  <si>
-    <t>DMU18-2</t>
-  </si>
-  <si>
-    <t>4617</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ST AMAND P H (3) </t>
-  </si>
-  <si>
-    <t>20/09/2026</t>
-  </si>
-  <si>
-    <t>13:00</t>
-  </si>
-  <si>
-    <t>MAURICE HUGOT</t>
-  </si>
-  <si>
-    <t>M9XEW737</t>
-  </si>
-  <si>
     <t>DMU13-8</t>
   </si>
   <si>
@@ -149,22 +176,46 @@
     <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (6) </t>
   </si>
   <si>
-    <t>Jules LADOUMEGUE</t>
-  </si>
-  <si>
-    <t>DMU15-2</t>
-  </si>
-  <si>
-    <t>8961</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ONNAING JA (3) </t>
-  </si>
-  <si>
-    <t>18:30</t>
-  </si>
-  <si>
-    <t>Daniel COLMONT</t>
+    <t>C.S. J MERCIER</t>
+  </si>
+  <si>
+    <t>PRM</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT - 1 (3) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BASKET CLUB PEVELE (4) </t>
+  </si>
+  <si>
+    <t>DFU18-2</t>
+  </si>
+  <si>
+    <t>6915</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USAC SOMAIN MARCHIENNES BASKETBALL (6) </t>
+  </si>
+  <si>
+    <t>10:30</t>
+  </si>
+  <si>
+    <t>DFU15-8</t>
+  </si>
+  <si>
+    <t>25654</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (1) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BASKET CLUB PEVELE (2) </t>
+  </si>
+  <si>
+    <t>17:00</t>
   </si>
   <si>
     <t>DM2</t>
@@ -188,61 +239,10 @@
     <t>29251</t>
   </si>
   <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (1) </t>
-  </si>
-  <si>
     <t xml:space="preserve">AULNOY VALENCIENNES S (2) </t>
   </si>
   <si>
     <t>14:00</t>
-  </si>
-  <si>
-    <t>PRM</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT - 1 (3) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BASKET CLUB PEVELE (4) </t>
-  </si>
-  <si>
-    <t>DFU18-2</t>
-  </si>
-  <si>
-    <t>6915</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (5) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">USAC SOMAIN MARCHIENNES BASKETBALL (6) </t>
-  </si>
-  <si>
-    <t>10:30</t>
-  </si>
-  <si>
-    <t>DFU15-8</t>
-  </si>
-  <si>
-    <t>25654</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BASKET CLUB PEVELE (2) </t>
-  </si>
-  <si>
-    <t>17:00</t>
-  </si>
-  <si>
-    <t>DXU9-8</t>
-  </si>
-  <si>
-    <t>29959</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ST AMAND P H (6) </t>
   </si>
 </sst>
 </file>
@@ -297,7 +297,7 @@
     <col min="4" max="4" width="45.765625" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="15.27734375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="5.65234375" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="16.3359375" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="14.37109375" customWidth="true" bestFit="true"/>
     <col min="8" max="8" width="10.9296875" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="6.83203125" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="7.4765625" customWidth="true" bestFit="true"/>
@@ -433,16 +433,16 @@
         <v>30</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G4" t="s" s="0">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H4" t="s" s="0">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I4" t="s" s="0">
         <v>19</v>
@@ -459,28 +459,28 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s" s="0">
         <v>30</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="F5" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="G5" t="s" s="0">
         <v>38</v>
       </c>
-      <c r="G5" t="s" s="0">
+      <c r="H5" t="s" s="0">
         <v>39</v>
-      </c>
-      <c r="H5" t="s" s="0">
-        <v>40</v>
       </c>
       <c r="I5" t="s" s="0">
         <v>19</v>
@@ -497,25 +497,25 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="B6" t="s" s="0">
         <v>41</v>
       </c>
-      <c r="B6" t="s" s="0">
+      <c r="C6" t="s" s="0">
         <v>42</v>
       </c>
-      <c r="C6" t="s" s="0">
+      <c r="D6" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="F6" t="s" s="0">
         <v>43</v>
       </c>
-      <c r="D6" t="s" s="0">
+      <c r="G6" t="s" s="0">
         <v>44</v>
-      </c>
-      <c r="E6" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="F6" t="s" s="0">
-        <v>25</v>
-      </c>
-      <c r="G6" t="s" s="0">
-        <v>45</v>
       </c>
       <c r="H6" t="s" s="0">
         <v>19</v>
@@ -535,16 +535,16 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="B7" t="s" s="0">
         <v>46</v>
       </c>
-      <c r="B7" t="s" s="0">
+      <c r="C7" t="s" s="0">
         <v>47</v>
       </c>
-      <c r="C7" t="s" s="0">
+      <c r="D7" t="s" s="0">
         <v>48</v>
-      </c>
-      <c r="D7" t="s" s="0">
-        <v>30</v>
       </c>
       <c r="E7" t="s" s="0">
         <v>16</v>
@@ -553,7 +553,7 @@
         <v>49</v>
       </c>
       <c r="G7" t="s" s="0">
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="H7" t="s" s="0">
         <v>19</v>
@@ -573,25 +573,25 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="B8" t="s" s="0">
         <v>51</v>
       </c>
-      <c r="B8" t="s" s="0">
+      <c r="C8" t="s" s="0">
         <v>52</v>
       </c>
-      <c r="C8" t="s" s="0">
+      <c r="D8" t="s" s="0">
         <v>53</v>
       </c>
-      <c r="D8" t="s" s="0">
+      <c r="E8" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="G8" t="s" s="0">
         <v>54</v>
-      </c>
-      <c r="E8" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="F8" t="s" s="0">
-        <v>55</v>
-      </c>
-      <c r="G8" t="s" s="0">
-        <v>26</v>
       </c>
       <c r="H8" t="s" s="0">
         <v>19</v>
@@ -611,25 +611,25 @@
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="B9" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="B9" t="s" s="0">
+      <c r="C9" t="s" s="0">
         <v>57</v>
       </c>
-      <c r="C9" t="s" s="0">
+      <c r="D9" t="s" s="0">
         <v>58</v>
       </c>
-      <c r="D9" t="s" s="0">
-        <v>59</v>
-      </c>
       <c r="E9" t="s" s="0">
         <v>16</v>
       </c>
       <c r="F9" t="s" s="0">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="G9" t="s" s="0">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="H9" t="s" s="0">
         <v>19</v>
@@ -649,25 +649,25 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="D10" t="s" s="0">
         <v>61</v>
       </c>
-      <c r="B10" t="s" s="0">
+      <c r="E10" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="F10" t="s" s="0">
         <v>62</v>
       </c>
-      <c r="C10" t="s" s="0">
-        <v>63</v>
-      </c>
-      <c r="D10" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="E10" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="F10" t="s" s="0">
-        <v>49</v>
-      </c>
       <c r="G10" t="s" s="0">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="H10" t="s" s="0">
         <v>19</v>
@@ -687,25 +687,25 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="C11" t="s" s="0">
         <v>65</v>
       </c>
-      <c r="B11" t="s" s="0">
+      <c r="D11" t="s" s="0">
         <v>66</v>
       </c>
-      <c r="C11" t="s" s="0">
+      <c r="E11" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="F11" t="s" s="0">
         <v>67</v>
       </c>
-      <c r="D11" t="s" s="0">
-        <v>68</v>
-      </c>
-      <c r="E11" t="s" s="0">
-        <v>37</v>
-      </c>
-      <c r="F11" t="s" s="0">
-        <v>69</v>
-      </c>
       <c r="G11" t="s" s="0">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="H11" t="s" s="0">
         <v>19</v>
@@ -725,25 +725,25 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="C12" t="s" s="0">
         <v>70</v>
       </c>
-      <c r="B12" t="s" s="0">
+      <c r="D12" t="s" s="0">
         <v>71</v>
       </c>
-      <c r="C12" t="s" s="0">
-        <v>58</v>
-      </c>
-      <c r="D12" t="s" s="0">
+      <c r="E12" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="F12" t="s" s="0">
         <v>72</v>
       </c>
-      <c r="E12" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="F12" t="s" s="0">
-        <v>73</v>
-      </c>
       <c r="G12" t="s" s="0">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="H12" t="s" s="0">
         <v>19</v>
@@ -763,25 +763,25 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
+        <v>73</v>
+      </c>
+      <c r="B13" t="s" s="0">
         <v>74</v>
       </c>
-      <c r="B13" t="s" s="0">
+      <c r="C13" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D13" t="s" s="0">
         <v>75</v>
       </c>
-      <c r="C13" t="s" s="0">
-        <v>67</v>
-      </c>
-      <c r="D13" t="s" s="0">
+      <c r="E13" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="F13" t="s" s="0">
         <v>76</v>
       </c>
-      <c r="E13" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="F13" t="s" s="0">
-        <v>31</v>
-      </c>
       <c r="G13" t="s" s="0">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="H13" t="s" s="0">
         <v>19</v>

</xml_diff>

<commit_message>
Mise a jour automatique 06/10/2026 13:29:13,13
</commit_message>
<xml_diff>
--- a/data/rencontres/rencontres.xlsx
+++ b/data/rencontres/rencontres.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="79">
   <si>
     <t>Division</t>
   </si>
@@ -50,175 +50,205 @@
     <t>Forfait 2</t>
   </si>
   <si>
+    <t>DXU9-8</t>
+  </si>
+  <si>
+    <t>30038</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (5) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BREBIERES BC (4) </t>
+  </si>
+  <si>
+    <t>10/10/2026</t>
+  </si>
+  <si>
+    <t>14:00</t>
+  </si>
+  <si>
+    <t>JEAN DEGROS</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Non</t>
+  </si>
+  <si>
+    <t>DMU13-8</t>
+  </si>
+  <si>
+    <t>27149</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (4) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CUINCY ASB (5) </t>
+  </si>
+  <si>
+    <t>15:30</t>
+  </si>
+  <si>
+    <t>DFU18-2</t>
+  </si>
+  <si>
+    <t>6985</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOUAI BASKET FEMININ - 3 (1) </t>
+  </si>
+  <si>
+    <t>17:00</t>
+  </si>
+  <si>
+    <t>AMILOISIRS</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAUDRY BC (14) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (1) </t>
+  </si>
+  <si>
+    <t>11/10/2026</t>
+  </si>
+  <si>
+    <t>DM2</t>
+  </si>
+  <si>
+    <t>660</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNION DECHY SIN BASKET - 3 (5) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT - 2 (4) </t>
+  </si>
+  <si>
+    <t>20:30</t>
+  </si>
+  <si>
+    <t>Jules LADOUMEGUE</t>
+  </si>
+  <si>
+    <t>DMU15-2</t>
+  </si>
+  <si>
+    <t>8998</t>
+  </si>
+  <si>
+    <t>Exempt</t>
+  </si>
+  <si>
+    <t>18:30</t>
+  </si>
+  <si>
     <t>DFU13-2</t>
   </si>
   <si>
-    <t>11266</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (5) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">ST AMAND P H (4) </t>
-  </si>
-  <si>
-    <t>03/10/2026</t>
-  </si>
-  <si>
-    <t>15:30</t>
-  </si>
-  <si>
-    <t>JEAN DEGROS</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Non</t>
+    <t>11273</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MARCQ EN BAROEUL ASJ (2) </t>
+  </si>
+  <si>
+    <t>SALLE LAZARO</t>
+  </si>
+  <si>
+    <t>96244FCY</t>
+  </si>
+  <si>
+    <t>DMU11-8</t>
+  </si>
+  <si>
+    <t>28493</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GAYANT BASKET (4) </t>
+  </si>
+  <si>
+    <t>Jean-Baptiste COROT</t>
+  </si>
+  <si>
+    <t>27BFVHNG</t>
   </si>
   <si>
     <t>PRM</t>
   </si>
   <si>
-    <t>64</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT - 1 (6) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">ST AMAND P H - 1 (5) </t>
-  </si>
-  <si>
-    <t>18:30</t>
-  </si>
-  <si>
-    <t>DM2</t>
-  </si>
-  <si>
-    <t>629</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT - 2 (5) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">SECLIN BC - 2 (2) </t>
-  </si>
-  <si>
-    <t>20:30</t>
-  </si>
-  <si>
-    <t>DMU13-8</t>
-  </si>
-  <si>
-    <t>27118</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BREBIERES BC (4) </t>
+    <t>89</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JEUNESSE BASKET CLUB AUBY - 1 (1) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT - 1 (4) </t>
+  </si>
+  <si>
+    <t>Michel DUJARDIN</t>
+  </si>
+  <si>
+    <t>DFU11-8</t>
+  </si>
+  <si>
+    <t>29305</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USAC SOMAIN MARCHIENNES BASKETBALL (3) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (2) </t>
+  </si>
+  <si>
+    <t>10:30</t>
+  </si>
+  <si>
+    <t>Léo LAGRANGE</t>
+  </si>
+  <si>
+    <t>DFU15-8</t>
+  </si>
+  <si>
+    <t>25708</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CUINCY ASB (2) </t>
   </si>
   <si>
     <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (3) </t>
   </si>
   <si>
-    <t>FRANCOIS ANACHE</t>
+    <t>Jean LENNE</t>
+  </si>
+  <si>
+    <t>GFQAAW8G</t>
   </si>
   <si>
     <t>DFU9-8</t>
   </si>
   <si>
-    <t>30818</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BEUVRAGES ASM (6) </t>
-  </si>
-  <si>
-    <t>Léo LAGRANGE</t>
-  </si>
-  <si>
-    <t>DXU9-8</t>
-  </si>
-  <si>
-    <t>30011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GAYANT BASKET (3) </t>
-  </si>
-  <si>
-    <t>04/10/2026</t>
-  </si>
-  <si>
-    <t>14:00</t>
-  </si>
-  <si>
-    <t>Jean-Baptiste COROT</t>
-  </si>
-  <si>
-    <t>DFU18-2</t>
-  </si>
-  <si>
-    <t>6961</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNION DECHY SIN BASKET (3) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (6) </t>
-  </si>
-  <si>
-    <t>10:30</t>
-  </si>
-  <si>
-    <t>C.S. J MERCIER</t>
+    <t>30825</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AULNOY VALENCIENNES S (7) </t>
+  </si>
+  <si>
+    <t>11:00</t>
   </si>
   <si>
     <t>DMU18-2</t>
   </si>
   <si>
-    <t>4664</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (4) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">HASNON BASKET - 2 (1) </t>
-  </si>
-  <si>
-    <t>DMU11-8</t>
-  </si>
-  <si>
-    <t>28463</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ASC DENAIN VOLTAIRE PORTE DU HAINAUT - 2 (2) </t>
-  </si>
-  <si>
-    <t>DMU15-2</t>
-  </si>
-  <si>
-    <t>8986</t>
-  </si>
-  <si>
-    <t>16:00</t>
-  </si>
-  <si>
-    <t>DFU11-8</t>
-  </si>
-  <si>
-    <t>29288</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OSTREVENT BASKET BALL EAA MONCHECOURT (4) </t>
-  </si>
-  <si>
-    <t>DFU15-8</t>
-  </si>
-  <si>
-    <t>25691</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OSTREVENT BASKET BALL EAA MONCHECOURT (6) </t>
-  </si>
-  <si>
-    <t>17:00</t>
+    <t>4689</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAMBRES BASKET CLUB - 2 (4) </t>
   </si>
 </sst>
 </file>
@@ -264,13 +294,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="8.1796875" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="9.91796875" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="11.29296875" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="33.890625" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="41.3671875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="37.88671875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="33.890625" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="15.27734375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="5.65234375" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="17.46875" customWidth="true" bestFit="true"/>
@@ -403,16 +433,16 @@
         <v>27</v>
       </c>
       <c r="C4" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s" s="0">
         <v>28</v>
       </c>
-      <c r="D4" t="s" s="0">
+      <c r="E4" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="F4" t="s" s="0">
         <v>29</v>
-      </c>
-      <c r="E4" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="F4" t="s" s="0">
-        <v>30</v>
       </c>
       <c r="G4" t="s" s="0">
         <v>18</v>
@@ -435,26 +465,24 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s" s="0">
         <v>31</v>
       </c>
-      <c r="B5" t="s" s="0">
+      <c r="C5" t="s" s="0">
         <v>32</v>
       </c>
-      <c r="C5" t="s" s="0">
+      <c r="D5" t="s" s="0">
         <v>33</v>
       </c>
-      <c r="D5" t="s" s="0">
+      <c r="E5" t="s" s="0">
         <v>34</v>
-      </c>
-      <c r="E5" t="s" s="0">
-        <v>16</v>
       </c>
       <c r="F5" t="s" s="0">
         <v>17</v>
       </c>
-      <c r="G5" t="s" s="0">
-        <v>35</v>
-      </c>
+      <c r="G5" s="0"/>
       <c r="H5" t="s" s="0">
         <v>19</v>
       </c>
@@ -473,25 +501,25 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B6" t="s" s="0">
         <v>36</v>
       </c>
-      <c r="B6" t="s" s="0">
+      <c r="C6" t="s" s="0">
         <v>37</v>
       </c>
-      <c r="C6" t="s" s="0">
+      <c r="D6" t="s" s="0">
         <v>38</v>
       </c>
-      <c r="D6" t="s" s="0">
-        <v>34</v>
-      </c>
       <c r="E6" t="s" s="0">
         <v>16</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="G6" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H6" t="s" s="0">
         <v>19</v>
@@ -511,26 +539,24 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>43</v>
+        <v>16</v>
       </c>
       <c r="F7" t="s" s="0">
         <v>44</v>
       </c>
-      <c r="G7" t="s" s="0">
-        <v>45</v>
-      </c>
+      <c r="G7" s="0"/>
       <c r="H7" t="s" s="0">
         <v>19</v>
       </c>
@@ -549,28 +575,28 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="B8" t="s" s="0">
         <v>46</v>
       </c>
-      <c r="B8" t="s" s="0">
+      <c r="C8" t="s" s="0">
         <v>47</v>
       </c>
-      <c r="C8" t="s" s="0">
+      <c r="D8" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="G8" t="s" s="0">
         <v>48</v>
       </c>
-      <c r="D8" t="s" s="0">
+      <c r="H8" t="s" s="0">
         <v>49</v>
-      </c>
-      <c r="E8" t="s" s="0">
-        <v>43</v>
-      </c>
-      <c r="F8" t="s" s="0">
-        <v>50</v>
-      </c>
-      <c r="G8" t="s" s="0">
-        <v>51</v>
-      </c>
-      <c r="H8" t="s" s="0">
-        <v>19</v>
       </c>
       <c r="I8" t="s" s="0">
         <v>19</v>
@@ -587,28 +613,28 @@
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>51</v>
+      </c>
+      <c r="C9" t="s" s="0">
         <v>52</v>
       </c>
-      <c r="B9" t="s" s="0">
+      <c r="D9" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="F9" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="G9" t="s" s="0">
         <v>53</v>
       </c>
-      <c r="C9" t="s" s="0">
+      <c r="H9" t="s" s="0">
         <v>54</v>
-      </c>
-      <c r="D9" t="s" s="0">
-        <v>55</v>
-      </c>
-      <c r="E9" t="s" s="0">
-        <v>43</v>
-      </c>
-      <c r="F9" t="s" s="0">
-        <v>50</v>
-      </c>
-      <c r="G9" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="H9" t="s" s="0">
-        <v>19</v>
       </c>
       <c r="I9" t="s" s="0">
         <v>19</v>
@@ -625,25 +651,25 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="B10" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="B10" t="s" s="0">
+      <c r="C10" t="s" s="0">
         <v>57</v>
-      </c>
-      <c r="C10" t="s" s="0">
-        <v>14</v>
       </c>
       <c r="D10" t="s" s="0">
         <v>58</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>43</v>
+        <v>16</v>
       </c>
       <c r="F10" t="s" s="0">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="G10" t="s" s="0">
-        <v>18</v>
+        <v>59</v>
       </c>
       <c r="H10" t="s" s="0">
         <v>19</v>
@@ -663,25 +689,25 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="F11" t="s" s="0">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G11" t="s" s="0">
-        <v>18</v>
+        <v>65</v>
       </c>
       <c r="H11" t="s" s="0">
         <v>19</v>
@@ -701,28 +727,28 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C12" t="s" s="0">
-        <v>34</v>
+        <v>68</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="E12" t="s" s="0">
         <v>16</v>
       </c>
       <c r="F12" t="s" s="0">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="G12" t="s" s="0">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="H12" t="s" s="0">
-        <v>19</v>
+        <v>71</v>
       </c>
       <c r="I12" t="s" s="0">
         <v>19</v>
@@ -739,22 +765,22 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>34</v>
+        <v>63</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="E13" t="s" s="0">
         <v>16</v>
       </c>
       <c r="F13" t="s" s="0">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="G13" t="s" s="0">
         <v>18</v>
@@ -772,6 +798,44 @@
         <v>19</v>
       </c>
       <c r="L13" t="s" s="0">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="D14" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="E14" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="F14" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="G14" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="H14" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="I14" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="J14" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="K14" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="L14" t="s" s="0">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise a jour automatique 06/10/2026 13:33:50,85
</commit_message>
<xml_diff>
--- a/data/rencontres/rencontres.xlsx
+++ b/data/rencontres/rencontres.xlsx
@@ -77,178 +77,178 @@
     <t>Non</t>
   </si>
   <si>
+    <t>DMU18-2</t>
+  </si>
+  <si>
+    <t>4689</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAMBRES BASKET CLUB - 2 (4) </t>
+  </si>
+  <si>
+    <t>18:30</t>
+  </si>
+  <si>
+    <t>DFU11-8</t>
+  </si>
+  <si>
+    <t>29305</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USAC SOMAIN MARCHIENNES BASKETBALL (3) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (2) </t>
+  </si>
+  <si>
+    <t>11/10/2026</t>
+  </si>
+  <si>
+    <t>10:30</t>
+  </si>
+  <si>
+    <t>Léo LAGRANGE</t>
+  </si>
+  <si>
+    <t>DM2</t>
+  </si>
+  <si>
+    <t>660</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNION DECHY SIN BASKET - 3 (5) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT - 2 (4) </t>
+  </si>
+  <si>
+    <t>20:30</t>
+  </si>
+  <si>
+    <t>Jules LADOUMEGUE</t>
+  </si>
+  <si>
+    <t>DFU15-8</t>
+  </si>
+  <si>
+    <t>25708</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CUINCY ASB (2) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (3) </t>
+  </si>
+  <si>
+    <t>17:00</t>
+  </si>
+  <si>
+    <t>Jean LENNE</t>
+  </si>
+  <si>
+    <t>GFQAAW8G</t>
+  </si>
+  <si>
+    <t>AMILOISIRS</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAUDRY BC (14) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (1) </t>
+  </si>
+  <si>
+    <t>DMU11-8</t>
+  </si>
+  <si>
+    <t>28493</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GAYANT BASKET (4) </t>
+  </si>
+  <si>
+    <t>Jean-Baptiste COROT</t>
+  </si>
+  <si>
+    <t>27BFVHNG</t>
+  </si>
+  <si>
+    <t>DFU13-2</t>
+  </si>
+  <si>
+    <t>11273</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MARCQ EN BAROEUL ASJ (2) </t>
+  </si>
+  <si>
+    <t>15:30</t>
+  </si>
+  <si>
+    <t>SALLE LAZARO</t>
+  </si>
+  <si>
+    <t>96244FCY</t>
+  </si>
+  <si>
+    <t>DMU15-2</t>
+  </si>
+  <si>
+    <t>8998</t>
+  </si>
+  <si>
+    <t>Exempt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (4) </t>
+  </si>
+  <si>
+    <t>PRM</t>
+  </si>
+  <si>
+    <t>89</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JEUNESSE BASKET CLUB AUBY - 1 (1) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT - 1 (4) </t>
+  </si>
+  <si>
+    <t>Michel DUJARDIN</t>
+  </si>
+  <si>
+    <t>DFU9-8</t>
+  </si>
+  <si>
+    <t>30825</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AULNOY VALENCIENNES S (7) </t>
+  </si>
+  <si>
+    <t>11:00</t>
+  </si>
+  <si>
+    <t>DFU18-2</t>
+  </si>
+  <si>
+    <t>6985</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOUAI BASKET FEMININ - 3 (1) </t>
+  </si>
+  <si>
     <t>DMU13-8</t>
   </si>
   <si>
     <t>27149</t>
   </si>
   <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (4) </t>
-  </si>
-  <si>
     <t xml:space="preserve">CUINCY ASB (5) </t>
-  </si>
-  <si>
-    <t>15:30</t>
-  </si>
-  <si>
-    <t>DFU18-2</t>
-  </si>
-  <si>
-    <t>6985</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DOUAI BASKET FEMININ - 3 (1) </t>
-  </si>
-  <si>
-    <t>17:00</t>
-  </si>
-  <si>
-    <t>AMILOISIRS</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAUDRY BC (14) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (1) </t>
-  </si>
-  <si>
-    <t>11/10/2026</t>
-  </si>
-  <si>
-    <t>DM2</t>
-  </si>
-  <si>
-    <t>660</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNION DECHY SIN BASKET - 3 (5) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT - 2 (4) </t>
-  </si>
-  <si>
-    <t>20:30</t>
-  </si>
-  <si>
-    <t>Jules LADOUMEGUE</t>
-  </si>
-  <si>
-    <t>DMU15-2</t>
-  </si>
-  <si>
-    <t>8998</t>
-  </si>
-  <si>
-    <t>Exempt</t>
-  </si>
-  <si>
-    <t>18:30</t>
-  </si>
-  <si>
-    <t>DFU13-2</t>
-  </si>
-  <si>
-    <t>11273</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MARCQ EN BAROEUL ASJ (2) </t>
-  </si>
-  <si>
-    <t>SALLE LAZARO</t>
-  </si>
-  <si>
-    <t>96244FCY</t>
-  </si>
-  <si>
-    <t>DMU11-8</t>
-  </si>
-  <si>
-    <t>28493</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GAYANT BASKET (4) </t>
-  </si>
-  <si>
-    <t>Jean-Baptiste COROT</t>
-  </si>
-  <si>
-    <t>27BFVHNG</t>
-  </si>
-  <si>
-    <t>PRM</t>
-  </si>
-  <si>
-    <t>89</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JEUNESSE BASKET CLUB AUBY - 1 (1) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT - 1 (4) </t>
-  </si>
-  <si>
-    <t>Michel DUJARDIN</t>
-  </si>
-  <si>
-    <t>DFU11-8</t>
-  </si>
-  <si>
-    <t>29305</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USAC SOMAIN MARCHIENNES BASKETBALL (3) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (2) </t>
-  </si>
-  <si>
-    <t>10:30</t>
-  </si>
-  <si>
-    <t>Léo LAGRANGE</t>
-  </si>
-  <si>
-    <t>DFU15-8</t>
-  </si>
-  <si>
-    <t>25708</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CUINCY ASB (2) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (3) </t>
-  </si>
-  <si>
-    <t>Jean LENNE</t>
-  </si>
-  <si>
-    <t>GFQAAW8G</t>
-  </si>
-  <si>
-    <t>DFU9-8</t>
-  </si>
-  <si>
-    <t>30825</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AULNOY VALENCIENNES S (7) </t>
-  </si>
-  <si>
-    <t>11:00</t>
-  </si>
-  <si>
-    <t>DMU18-2</t>
-  </si>
-  <si>
-    <t>4689</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LAMBRES BASKET CLUB - 2 (4) </t>
   </si>
 </sst>
 </file>
@@ -395,16 +395,16 @@
         <v>22</v>
       </c>
       <c r="C3" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="D3" t="s" s="0">
+      <c r="E3" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="F3" t="s" s="0">
         <v>24</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s" s="0">
-        <v>25</v>
       </c>
       <c r="G3" t="s" s="0">
         <v>18</v>
@@ -427,25 +427,25 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="B4" t="s" s="0">
         <v>26</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="C4" t="s" s="0">
         <v>27</v>
-      </c>
-      <c r="C4" t="s" s="0">
-        <v>14</v>
       </c>
       <c r="D4" t="s" s="0">
         <v>28</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G4" t="s" s="0">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="H4" t="s" s="0">
         <v>19</v>
@@ -465,24 +465,26 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="G5" s="0"/>
+        <v>36</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>37</v>
+      </c>
       <c r="H5" t="s" s="0">
         <v>19</v>
       </c>
@@ -501,28 +503,28 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E6" t="s" s="0">
         <v>16</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G6" t="s" s="0">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="H6" t="s" s="0">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="I6" t="s" s="0">
         <v>19</v>
@@ -539,22 +541,22 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="F7" t="s" s="0">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="G7" s="0"/>
       <c r="H7" t="s" s="0">
@@ -575,28 +577,28 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="D8" t="s" s="0">
         <v>14</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="F8" t="s" s="0">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="G8" t="s" s="0">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="H8" t="s" s="0">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="I8" t="s" s="0">
         <v>19</v>
@@ -613,28 +615,28 @@
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D9" t="s" s="0">
         <v>14</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="F9" t="s" s="0">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="G9" t="s" s="0">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="H9" t="s" s="0">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="I9" t="s" s="0">
         <v>19</v>
@@ -651,26 +653,24 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="E10" t="s" s="0">
         <v>16</v>
       </c>
       <c r="F10" t="s" s="0">
-        <v>39</v>
-      </c>
-      <c r="G10" t="s" s="0">
-        <v>59</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="G10" s="0"/>
       <c r="H10" t="s" s="0">
         <v>19</v>
       </c>
@@ -689,25 +689,25 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="F11" t="s" s="0">
-        <v>64</v>
+        <v>36</v>
       </c>
       <c r="G11" t="s" s="0">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="H11" t="s" s="0">
         <v>19</v>
@@ -727,28 +727,28 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C12" t="s" s="0">
-        <v>68</v>
+        <v>28</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E12" t="s" s="0">
         <v>16</v>
       </c>
       <c r="F12" t="s" s="0">
-        <v>29</v>
+        <v>72</v>
       </c>
       <c r="G12" t="s" s="0">
-        <v>70</v>
+        <v>18</v>
       </c>
       <c r="H12" t="s" s="0">
-        <v>71</v>
+        <v>19</v>
       </c>
       <c r="I12" t="s" s="0">
         <v>19</v>
@@ -765,22 +765,22 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>63</v>
+        <v>14</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E13" t="s" s="0">
         <v>16</v>
       </c>
       <c r="F13" t="s" s="0">
-        <v>75</v>
+        <v>42</v>
       </c>
       <c r="G13" t="s" s="0">
         <v>18</v>
@@ -809,7 +809,7 @@
         <v>77</v>
       </c>
       <c r="C14" t="s" s="0">
-        <v>14</v>
+        <v>63</v>
       </c>
       <c r="D14" t="s" s="0">
         <v>78</v>
@@ -818,7 +818,7 @@
         <v>16</v>
       </c>
       <c r="F14" t="s" s="0">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="G14" t="s" s="0">
         <v>18</v>

</xml_diff>

<commit_message>
Mise a jour automatique 13/10/2026 20:31:25,22
</commit_message>
<xml_diff>
--- a/data/rencontres/rencontres.xlsx
+++ b/data/rencontres/rencontres.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="73">
   <si>
     <t>Division</t>
   </si>
@@ -50,205 +50,187 @@
     <t>Forfait 2</t>
   </si>
   <si>
+    <t>DM2</t>
+  </si>
+  <si>
+    <t>689</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CUINCY ASB (3) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT - 2 (4) </t>
+  </si>
+  <si>
+    <t>17/10/2026</t>
+  </si>
+  <si>
+    <t>18:30</t>
+  </si>
+  <si>
+    <t>Jean LENNE</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Non</t>
+  </si>
+  <si>
+    <t>DMU13-8</t>
+  </si>
+  <si>
+    <t>27178</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DORIGNIES DOUAI AAE (1) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (4) </t>
+  </si>
+  <si>
+    <t>15:30</t>
+  </si>
+  <si>
+    <t>Théo BOUTON</t>
+  </si>
+  <si>
+    <t>DMU18-2</t>
+  </si>
+  <si>
+    <t>4712</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BRILLON BASKET COMPETITION ET LOISIR (4) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (5) </t>
+  </si>
+  <si>
+    <t>17:00</t>
+  </si>
+  <si>
+    <t>INTERCOMMUNALE</t>
+  </si>
+  <si>
+    <t>DFU13-2</t>
+  </si>
+  <si>
+    <t>11278</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CYSOING SAINGHIN BOUVINES BASKET (2) </t>
+  </si>
+  <si>
+    <t>COMPLEXE SPORTIF</t>
+  </si>
+  <si>
     <t>DXU9-8</t>
   </si>
   <si>
-    <t>30038</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (5) </t>
+    <t>30067</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ORCHESIEN B C - 3 (6) </t>
+  </si>
+  <si>
+    <t>18/10/2026</t>
+  </si>
+  <si>
+    <t>09:30</t>
+  </si>
+  <si>
+    <t>LEO LAGRANGE</t>
+  </si>
+  <si>
+    <t>C3TQW7KM</t>
+  </si>
+  <si>
+    <t>DFU9-8</t>
+  </si>
+  <si>
+    <t>30835</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST AMAND P H (4) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (2) </t>
+  </si>
+  <si>
+    <t>14:00</t>
+  </si>
+  <si>
+    <t>du MOULIN BLANC</t>
+  </si>
+  <si>
+    <t>L4KFXZUQ</t>
+  </si>
+  <si>
+    <t>PRM</t>
+  </si>
+  <si>
+    <t>112</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OSTREVENT BASKET BALL EAA MONCHECOURT - 2 (1) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT - 1 (5) </t>
+  </si>
+  <si>
+    <t>16:00</t>
+  </si>
+  <si>
+    <t>MUNICIPALE COQUELET</t>
+  </si>
+  <si>
+    <t>DFU11-8</t>
+  </si>
+  <si>
+    <t>29323</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BREBIERES BC (6) </t>
+  </si>
+  <si>
+    <t>JEAN DEGROS</t>
+  </si>
+  <si>
+    <t>DMU11-8</t>
+  </si>
+  <si>
+    <t>28523</t>
+  </si>
+  <si>
+    <t>DFU15-8</t>
+  </si>
+  <si>
+    <t>25726</t>
   </si>
   <si>
     <t xml:space="preserve">BREBIERES BC (4) </t>
   </si>
   <si>
-    <t>10/10/2026</t>
-  </si>
-  <si>
-    <t>14:00</t>
-  </si>
-  <si>
-    <t>JEAN DEGROS</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Non</t>
-  </si>
-  <si>
-    <t>DMU18-2</t>
-  </si>
-  <si>
-    <t>4689</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LAMBRES BASKET CLUB - 2 (4) </t>
-  </si>
-  <si>
-    <t>18:30</t>
-  </si>
-  <si>
-    <t>DFU11-8</t>
-  </si>
-  <si>
-    <t>29305</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USAC SOMAIN MARCHIENNES BASKETBALL (3) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (2) </t>
-  </si>
-  <si>
-    <t>11/10/2026</t>
-  </si>
-  <si>
-    <t>10:30</t>
-  </si>
-  <si>
-    <t>Léo LAGRANGE</t>
-  </si>
-  <si>
-    <t>DM2</t>
-  </si>
-  <si>
-    <t>660</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNION DECHY SIN BASKET - 3 (5) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT - 2 (4) </t>
+    <t>DMU15-2</t>
+  </si>
+  <si>
+    <t>9010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST AMAND P H (5) </t>
+  </si>
+  <si>
+    <t>DFU18-2</t>
+  </si>
+  <si>
+    <t>7011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (6) </t>
   </si>
   <si>
     <t>20:30</t>
-  </si>
-  <si>
-    <t>Jules LADOUMEGUE</t>
-  </si>
-  <si>
-    <t>DFU15-8</t>
-  </si>
-  <si>
-    <t>25708</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CUINCY ASB (2) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (3) </t>
-  </si>
-  <si>
-    <t>17:00</t>
-  </si>
-  <si>
-    <t>Jean LENNE</t>
-  </si>
-  <si>
-    <t>GFQAAW8G</t>
-  </si>
-  <si>
-    <t>AMILOISIRS</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAUDRY BC (14) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (1) </t>
-  </si>
-  <si>
-    <t>DMU11-8</t>
-  </si>
-  <si>
-    <t>28493</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GAYANT BASKET (4) </t>
-  </si>
-  <si>
-    <t>Jean-Baptiste COROT</t>
-  </si>
-  <si>
-    <t>27BFVHNG</t>
-  </si>
-  <si>
-    <t>DFU13-2</t>
-  </si>
-  <si>
-    <t>11273</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MARCQ EN BAROEUL ASJ (2) </t>
-  </si>
-  <si>
-    <t>15:30</t>
-  </si>
-  <si>
-    <t>SALLE LAZARO</t>
-  </si>
-  <si>
-    <t>96244FCY</t>
-  </si>
-  <si>
-    <t>DMU15-2</t>
-  </si>
-  <si>
-    <t>8998</t>
-  </si>
-  <si>
-    <t>Exempt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (4) </t>
-  </si>
-  <si>
-    <t>PRM</t>
-  </si>
-  <si>
-    <t>89</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JEUNESSE BASKET CLUB AUBY - 1 (1) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT - 1 (4) </t>
-  </si>
-  <si>
-    <t>Michel DUJARDIN</t>
-  </si>
-  <si>
-    <t>DFU9-8</t>
-  </si>
-  <si>
-    <t>30825</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AULNOY VALENCIENNES S (7) </t>
-  </si>
-  <si>
-    <t>11:00</t>
-  </si>
-  <si>
-    <t>DFU18-2</t>
-  </si>
-  <si>
-    <t>6985</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DOUAI BASKET FEMININ - 3 (1) </t>
-  </si>
-  <si>
-    <t>DMU13-8</t>
-  </si>
-  <si>
-    <t>27149</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CUINCY ASB (5) </t>
   </si>
 </sst>
 </file>
@@ -294,16 +276,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="9.91796875" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="8.1796875" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="11.29296875" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="37.88671875" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="33.890625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="43.93359375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="43.93359375" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="15.27734375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="5.65234375" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="17.46875" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="19.5390625" customWidth="true" bestFit="true"/>
     <col min="8" max="8" width="10.9296875" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="6.83203125" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="7.4765625" customWidth="true" bestFit="true"/>
@@ -395,19 +377,19 @@
         <v>22</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E3" t="s" s="0">
         <v>16</v>
       </c>
       <c r="F3" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G3" t="s" s="0">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="H3" t="s" s="0">
         <v>19</v>
@@ -427,25 +409,25 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G4" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H4" t="s" s="0">
         <v>19</v>
@@ -465,25 +447,25 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E5" t="s" s="0">
         <v>16</v>
       </c>
       <c r="F5" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="G5" t="s" s="0">
         <v>36</v>
-      </c>
-      <c r="G5" t="s" s="0">
-        <v>37</v>
       </c>
       <c r="H5" t="s" s="0">
         <v>19</v>
@@ -503,28 +485,28 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="B6" t="s" s="0">
         <v>38</v>
       </c>
-      <c r="B6" t="s" s="0">
+      <c r="C6" t="s" s="0">
         <v>39</v>
       </c>
-      <c r="C6" t="s" s="0">
+      <c r="D6" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E6" t="s" s="0">
         <v>40</v>
       </c>
-      <c r="D6" t="s" s="0">
+      <c r="F6" t="s" s="0">
         <v>41</v>
       </c>
-      <c r="E6" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="F6" t="s" s="0">
+      <c r="G6" t="s" s="0">
         <v>42</v>
       </c>
-      <c r="G6" t="s" s="0">
+      <c r="H6" t="s" s="0">
         <v>43</v>
-      </c>
-      <c r="H6" t="s" s="0">
-        <v>44</v>
       </c>
       <c r="I6" t="s" s="0">
         <v>19</v>
@@ -541,26 +523,28 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="B7" t="s" s="0">
         <v>45</v>
       </c>
-      <c r="B7" t="s" s="0">
+      <c r="C7" t="s" s="0">
         <v>46</v>
       </c>
-      <c r="C7" t="s" s="0">
+      <c r="D7" t="s" s="0">
         <v>47</v>
       </c>
-      <c r="D7" t="s" s="0">
+      <c r="E7" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="F7" t="s" s="0">
         <v>48</v>
       </c>
-      <c r="E7" t="s" s="0">
-        <v>29</v>
-      </c>
-      <c r="F7" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="G7" s="0"/>
+      <c r="G7" t="s" s="0">
+        <v>49</v>
+      </c>
       <c r="H7" t="s" s="0">
-        <v>19</v>
+        <v>50</v>
       </c>
       <c r="I7" t="s" s="0">
         <v>19</v>
@@ -577,28 +561,28 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>14</v>
+        <v>54</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="F8" t="s" s="0">
-        <v>17</v>
+        <v>55</v>
       </c>
       <c r="G8" t="s" s="0">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="H8" t="s" s="0">
-        <v>53</v>
+        <v>19</v>
       </c>
       <c r="I8" t="s" s="0">
         <v>19</v>
@@ -615,28 +599,28 @@
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>14</v>
+        <v>59</v>
       </c>
       <c r="E9" t="s" s="0">
         <v>16</v>
       </c>
       <c r="F9" t="s" s="0">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="G9" t="s" s="0">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H9" t="s" s="0">
-        <v>59</v>
+        <v>19</v>
       </c>
       <c r="I9" t="s" s="0">
         <v>19</v>
@@ -653,24 +637,26 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
+        <v>61</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>62</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="F10" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="G10" t="s" s="0">
         <v>60</v>
       </c>
-      <c r="B10" t="s" s="0">
-        <v>61</v>
-      </c>
-      <c r="C10" t="s" s="0">
-        <v>62</v>
-      </c>
-      <c r="D10" t="s" s="0">
-        <v>63</v>
-      </c>
-      <c r="E10" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="F10" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="G10" s="0"/>
       <c r="H10" t="s" s="0">
         <v>19</v>
       </c>
@@ -689,25 +675,25 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="B11" t="s" s="0">
         <v>64</v>
       </c>
-      <c r="B11" t="s" s="0">
+      <c r="C11" t="s" s="0">
+        <v>47</v>
+      </c>
+      <c r="D11" t="s" s="0">
         <v>65</v>
       </c>
-      <c r="C11" t="s" s="0">
-        <v>66</v>
-      </c>
-      <c r="D11" t="s" s="0">
-        <v>67</v>
-      </c>
       <c r="E11" t="s" s="0">
         <v>16</v>
       </c>
       <c r="F11" t="s" s="0">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G11" t="s" s="0">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="H11" t="s" s="0">
         <v>19</v>
@@ -727,25 +713,25 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C12" t="s" s="0">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E12" t="s" s="0">
         <v>16</v>
       </c>
       <c r="F12" t="s" s="0">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="G12" t="s" s="0">
-        <v>18</v>
+        <v>60</v>
       </c>
       <c r="H12" t="s" s="0">
         <v>19</v>
@@ -765,25 +751,25 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>14</v>
+        <v>71</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>75</v>
+        <v>53</v>
       </c>
       <c r="E13" t="s" s="0">
         <v>16</v>
       </c>
       <c r="F13" t="s" s="0">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="G13" t="s" s="0">
-        <v>18</v>
+        <v>60</v>
       </c>
       <c r="H13" t="s" s="0">
         <v>19</v>
@@ -798,44 +784,6 @@
         <v>19</v>
       </c>
       <c r="L13" t="s" s="0">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s" s="0">
-        <v>76</v>
-      </c>
-      <c r="B14" t="s" s="0">
-        <v>77</v>
-      </c>
-      <c r="C14" t="s" s="0">
-        <v>63</v>
-      </c>
-      <c r="D14" t="s" s="0">
-        <v>78</v>
-      </c>
-      <c r="E14" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="F14" t="s" s="0">
-        <v>57</v>
-      </c>
-      <c r="G14" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="H14" t="s" s="0">
-        <v>19</v>
-      </c>
-      <c r="I14" t="s" s="0">
-        <v>19</v>
-      </c>
-      <c r="J14" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="K14" t="s" s="0">
-        <v>19</v>
-      </c>
-      <c r="L14" t="s" s="0">
         <v>20</v>
       </c>
     </row>

</xml_diff>